<commit_message>
Nuova intestazione; sei contenitori tematici al posto dei tre livelli
Le tre partite esistenti passano in 'Per iniziare'; i fogli usano la
colonna 'contenitore' (i vecchi fogli con 'livello' restano accettati).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JM4otbn7ACBNqb6AC9EfAs
</commit_message>
<xml_diff>
--- a/fogli/modello-sondaggio.xlsx
+++ b/fogli/modello-sondaggio.xlsx
@@ -225,9 +225,14 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>Cheat Sheet</author>
+    <author>Gioco a indizi</author>
   </authors>
   <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Scegli il contenitore dal menu a tendina; uguale su tutte le righe.</t>
+      </text>
+    </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <t>{{parola}} = indizio da cliccare
@@ -535,7 +540,7 @@
   <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -549,7 +554,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>livello</t>
+          <t>contenitore</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -785,8 +790,8 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"1 - Base,2 - Intermedio,3 - Avanzato"</formula1>
+    <dataValidation sqref="A2:A11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Contenitore" error="Scegli uno dei contenitori dal menu." type="list">
+      <formula1>"Per iniziare,Identificazione e classificazione,Tensioni e deformazioni,Filtrazione e consolidazione,Comportamento meccanico,Prove di laboratorio"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -800,7 +805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -878,132 +883,139 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>livello: 1 - Base, 2 - Intermedio o 3 - Avanzato (menu a tendina). sondaggio: titolo breve (es. Tensioni efficaci), uguale su tutte le righe.</t>
+          <t>contenitore: l'argomento in cui compare il sondaggio (menu a tendina), uguale su tutte le righe: Per iniziare; Identificazione e classificazione; Tensioni e deformazioni; Filtrazione e consolidazione; Comportamento meccanico; Prove di laboratorio.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>risposte alternative: sinonimi accettati, separati da ; (accenti, maiuscole e piccoli refusi sono già tollerati).</t>
+          <t>sondaggio: titolo breve (es. Tensioni efficaci), uguale su tutte le righe.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
+          <t>risposte alternative: sinonimi accettati, separati da ; (accenti, maiuscole e piccoli refusi sono già tollerati).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
           <t>nota didattica: mostrata dopo la risposta. fonte: riferimento bibliografico o normativo.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr"/>
-    </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Caricamento</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Nella pagina del gioco apri 'Aggiungi sondaggi', scegli il file .xlsx (o .csv con le stesse colonne): la pagina controlla le regole e segnala eventuali errori riga per riga.</t>
-        </is>
-      </c>
-    </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr"/>
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Nella pagina del gioco apri 'Scarica o aggiungi sondaggi' e scegli il file .xlsx (o .csv con le stesse colonne): la pagina controlla le regole e segnala eventuali errori riga per riga.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Esempio di riga compilata (indizio A di 'Tensioni efficaci')</t>
-        </is>
-      </c>
+      <c r="A18" s="7" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>livello</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Esempio di riga compilata</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>contenitore</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>sondaggio</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>codice</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>domanda</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>risposta canonica</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>risposte alternative</t>
         </is>
       </c>
-      <c r="G19" s="8" t="inlineStr">
+      <c r="G20" s="8" t="inlineStr">
         <is>
           <t>nota didattica</t>
         </is>
       </c>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="H20" s="8" t="inlineStr">
         <is>
           <t>fonte</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>1 - Base</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Per iniziare</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Tensioni efficaci</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>Quale ingegnere, autore di Erdbaumechanik nel 1925, è considerato il padre della {{geotecnica}} moderna e ha formulato la teoria della {{consolidazione}} monodimensionale?</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E21" s="9" t="inlineStr">
         <is>
           <t>Terzaghi</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>karl terzaghi; karl von terzaghi; k terzaghi</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="G21" s="9" t="inlineStr">
         <is>
           <t>Karl Terzaghi (Praga 1883 – Winchester 1963). Erdbaumechanik auf bodenphysikalischer Grundlage (Vienna, 1925) segna la nascita della meccanica delle terre come disciplina autonoma.</t>
         </is>
       </c>
-      <c r="H20" s="9" t="inlineStr">
-        <is>
-          <t>Terzaghi K. (1925), Erdbaumechanik auf bodenphysikalischer Grundlage, Deuticke, Vienna</t>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>e.g., Berardi R., Fondamenti di geotecnica, Città studi edizioni</t>
         </is>
       </c>
     </row>

</xml_diff>